<commit_message>
chore(assets): track the Blue logo vector source and refresh the workbooks
blue_logo_vector.svg is the source the inline markup in
AnimatedBlueLogo.tsx was traced from — keeping it in the repo means the
logo can be re-cut without hunting for the original file.

dondathang.xlsx stays tracked on purpose: app.go resolves it with
resolveRepoFile and every run opens it in place, so a checkout without it
cannot process anything. It will keep showing up as modified after each
run — that is the workbook being written to, not a change to review.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\code py\Xử lý đơn hàng\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CC9748-E33B-42F6-864A-439D20687879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C76FFB-6734-4EEA-B8FF-5A1D2A024232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3315" yWindow="1650" windowWidth="23625" windowHeight="13290" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MaKH" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3946" uniqueCount="2835">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3955" uniqueCount="2851">
   <si>
     <t>HỆ THÔNG</t>
   </si>
@@ -8146,9 +8146,6 @@
     <t>[TopValue]TúinướcxảvảiBluedạngtúi2.1L/3.2L(2mùihương),Túi3.2L-Thanhxuân</t>
   </si>
   <si>
-    <t>NướcRửaChénBátBlueChiếtXuấtGạo/ĐậuXanhTúi2.1L–SạchBóngDầuMỡ,KhửMùi,DịuNhẹ,ChiếtxuấtGạo</t>
-  </si>
-  <si>
     <t>[TopValue]ChaithảbồncầutoiletChungBlue180g,Hươngcam</t>
   </si>
   <si>
@@ -8176,9 +8173,6 @@
     <t>[TopValue]NướcgiặtBluekhángkhuẩntúi3,2LMuốihồngHimalaya</t>
   </si>
   <si>
-    <t>NướcRửaChénbátBlueChiếtXuấtGạo&amp;ĐậuXanh800ml/1200ml–SạchBóng,AnToànChoTay,HươngThơmDễChịu,Gạo1.2L</t>
-  </si>
-  <si>
     <t>[TopValue]NướcxảvảiBluethanhxuân2,1L,</t>
   </si>
   <si>
@@ -8236,12 +8230,6 @@
     <t>Column2</t>
   </si>
   <si>
-    <t>[Top Value] Nước rửa chén Blue dạng túi nhiều mùi hươ ng (800g /1.2L/ 2.1L / 3.2L), 800g - Hương gạo</t>
-  </si>
-  <si>
-    <t>[Top Value] Túi Nước Giặt BLue dạng túi/can nhiều mùi hương, Túi 2.1L - Nước hoa</t>
-  </si>
-  <si>
     <t>[TopValue]ChaithảbồncầuSmileMomCH34màutím,Ngẫunhiên</t>
   </si>
   <si>
@@ -8336,9 +8324,6 @@
   </si>
   <si>
     <t>TP32781</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Viên tẩy Toilet Blue hương Ngàn hoa 300g </t>
   </si>
   <si>
     <t>[TopValue]NướcgiặtBeCleanCH50hươngphấnhồng3,6L(can),Phấnhồng-Can3.6L</t>
@@ -8632,6 +8617,69 @@
   </si>
   <si>
     <t>6-8 Đường Số 17, Phường Tân Hưng, Tp.HCM,VNM</t>
+  </si>
+  <si>
+    <t>TP32873</t>
+  </si>
+  <si>
+    <t>Bột tẩy đa năng Blue 300g</t>
+  </si>
+  <si>
+    <t>TP32651_02</t>
+  </si>
+  <si>
+    <t>Viên giặt xả Blue Hoa bạch trà 10.5g x 20v</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcgiặtBLUECH22loạisạchvếtbẩntốthơngấp2lầnchỉtrong1bướcgiặt800gNew,Ngẫunhiên</t>
+  </si>
+  <si>
+    <t>[TopValue]TúinướcgiặtBlueThảomộcCH443.6LNew,Thảomộc-Túi3.6L</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcgiặtđồlótBluechai510gNew,510g</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcrửachénBlueCH191200mlhươngĐậuxanhNew,Ngẫunhiên</t>
+  </si>
+  <si>
+    <t>[TopValue]BộttẩylồngmáygiặtSmileMom450gCH31vệsinhtiệndụngNew,Ngẫunhiên</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcrửachénBLUECH212.1Lhươngđậuxanhcótácdụngđánhbaydầumỡ,vếtbẩncứngđầuNew,Đậuxanh-2.1L</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcrửachénBluedạngtúinhiềumùihương(800g/1.2L/2.1L/3.2L)New,800g-Hươnggạo</t>
+  </si>
+  <si>
+    <t>[TopValue]ChaithảbồncầuSmileMomCH34màutímNew,Ngẫunhiên</t>
+  </si>
+  <si>
+    <t>[TopValue]BộtgiặtSmileMomCH37800gNew,800g</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcxảvảiBlueCH14túi3.2LHươnghươngthảothơmmátNew,Thanhthảo-Túi3.2L</t>
+  </si>
+  <si>
+    <t>[TopValue]TúiNướcGiặtBLuedạngtúi/cannhiềumùihươngNew,Túi2.1L-Nướchoa</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcrửachénBlueCH20túi2.1LhươnggạoNew,Hươnggạo-Túi2.1L</t>
+  </si>
+  <si>
+    <t>[TopValue]TúinướcgiặtBLueCH42túi2.1LThảomộcNew,Ngẫunhiên</t>
+  </si>
+  <si>
+    <t>[TopValue]TúinướcgiặtBLUECH433.6LhươngnướchoaNew,3,6l</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcrửachénBlueCH18hươnggạo1200mlNew,Ngẫunhiên</t>
+  </si>
+  <si>
+    <t>[TopValue]NướcgiặtBecleankhángkhuẩnHươngBiển2,1kgNew,2,1kg</t>
+  </si>
+  <si>
+    <t>Viên tẩy Toilet Blue 300g (6 viên x 50 g)</t>
   </si>
 </sst>
 </file>
@@ -11251,10 +11299,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>2809</v>
+        <v>2804</v>
       </c>
       <c r="C3" t="s">
-        <v>2811</v>
+        <v>2806</v>
       </c>
     </row>
     <row r="4" spans="1:4" hidden="1">
@@ -11262,10 +11310,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>2787</v>
+        <v>2782</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>2786</v>
+        <v>2781</v>
       </c>
     </row>
     <row r="5" spans="1:4" hidden="1">
@@ -12417,10 +12465,10 @@
         <v>83</v>
       </c>
       <c r="B109" t="s">
-        <v>2830</v>
+        <v>2825</v>
       </c>
       <c r="C109" s="20" t="s">
-        <v>2831</v>
+        <v>2826</v>
       </c>
     </row>
     <row r="110" spans="1:3" hidden="1">
@@ -12428,10 +12476,10 @@
         <v>83</v>
       </c>
       <c r="B110" t="s">
-        <v>2832</v>
+        <v>2827</v>
       </c>
       <c r="C110" s="20" t="s">
-        <v>2833</v>
+        <v>2828</v>
       </c>
     </row>
     <row r="111" spans="1:3" hidden="1">
@@ -12818,7 +12866,7 @@
         <v>188</v>
       </c>
       <c r="D139" t="s">
-        <v>2834</v>
+        <v>2829</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -14036,7 +14084,7 @@
         <v>362</v>
       </c>
       <c r="D226" t="s">
-        <v>2819</v>
+        <v>2814</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -14372,7 +14420,7 @@
         <v>410</v>
       </c>
       <c r="D250" t="s">
-        <v>2733</v>
+        <v>2729</v>
       </c>
     </row>
     <row r="251" spans="1:4">
@@ -14694,7 +14742,7 @@
         <v>456</v>
       </c>
       <c r="D273" t="s">
-        <v>2820</v>
+        <v>2815</v>
       </c>
     </row>
     <row r="274" spans="1:4">
@@ -14722,7 +14770,7 @@
         <v>460</v>
       </c>
       <c r="D275" t="s">
-        <v>2785</v>
+        <v>2780</v>
       </c>
     </row>
     <row r="276" spans="1:4">
@@ -15044,7 +15092,7 @@
         <v>502</v>
       </c>
       <c r="D298" t="s">
-        <v>2751</v>
+        <v>2747</v>
       </c>
     </row>
     <row r="299" spans="1:4">
@@ -15058,7 +15106,7 @@
         <v>504</v>
       </c>
       <c r="D299" t="s">
-        <v>2821</v>
+        <v>2816</v>
       </c>
     </row>
     <row r="300" spans="1:4">
@@ -16281,7 +16329,7 @@
         <v>704</v>
       </c>
       <c r="C406" s="6" t="s">
-        <v>2774</v>
+        <v>2769</v>
       </c>
     </row>
     <row r="407" spans="1:3" hidden="1">
@@ -16369,7 +16417,7 @@
         <v>717</v>
       </c>
       <c r="C414" s="10" t="s">
-        <v>2757</v>
+        <v>2752</v>
       </c>
     </row>
     <row r="415" spans="1:3" hidden="1">
@@ -16446,7 +16494,7 @@
         <v>730</v>
       </c>
       <c r="C421" t="s">
-        <v>2756</v>
+        <v>2751</v>
       </c>
     </row>
     <row r="422" spans="1:3" hidden="1">
@@ -17139,13 +17187,13 @@
         <v>848</v>
       </c>
       <c r="B484" s="5" t="s">
-        <v>2828</v>
+        <v>2823</v>
       </c>
       <c r="C484" s="6" t="s">
-        <v>2828</v>
+        <v>2823</v>
       </c>
       <c r="D484" t="s">
-        <v>2829</v>
+        <v>2824</v>
       </c>
     </row>
     <row r="485" spans="1:4" hidden="1">
@@ -17153,13 +17201,13 @@
         <v>848</v>
       </c>
       <c r="B485" s="5" t="s">
-        <v>2827</v>
+        <v>2822</v>
       </c>
       <c r="C485" s="6" t="s">
-        <v>2827</v>
+        <v>2822</v>
       </c>
       <c r="D485" t="s">
-        <v>2826</v>
+        <v>2821</v>
       </c>
     </row>
     <row r="486" spans="1:4" hidden="1">
@@ -17167,13 +17215,13 @@
         <v>848</v>
       </c>
       <c r="B486" s="5" t="s">
-        <v>2815</v>
+        <v>2810</v>
       </c>
       <c r="C486" s="6" t="s">
-        <v>2815</v>
+        <v>2810</v>
       </c>
       <c r="D486" t="s">
-        <v>2816</v>
+        <v>2811</v>
       </c>
     </row>
     <row r="487" spans="1:4" hidden="1">
@@ -17181,10 +17229,10 @@
         <v>848</v>
       </c>
       <c r="B487" s="5" t="s">
-        <v>2755</v>
+        <v>2750</v>
       </c>
       <c r="C487" s="6" t="s">
-        <v>2755</v>
+        <v>2750</v>
       </c>
     </row>
     <row r="488" spans="1:4" hidden="1">
@@ -17192,13 +17240,13 @@
         <v>848</v>
       </c>
       <c r="B488" s="5" t="s">
-        <v>2777</v>
+        <v>2772</v>
       </c>
       <c r="C488" s="6" t="s">
-        <v>2777</v>
+        <v>2772</v>
       </c>
       <c r="D488" t="s">
-        <v>2778</v>
+        <v>2773</v>
       </c>
     </row>
     <row r="489" spans="1:4" hidden="1">
@@ -17206,13 +17254,13 @@
         <v>848</v>
       </c>
       <c r="B489" s="5" t="s">
-        <v>2775</v>
+        <v>2770</v>
       </c>
       <c r="C489" s="6" t="s">
-        <v>2775</v>
+        <v>2770</v>
       </c>
       <c r="D489" t="s">
-        <v>2776</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="490" spans="1:4" hidden="1">
@@ -17220,13 +17268,13 @@
         <v>848</v>
       </c>
       <c r="B490" s="5" t="s">
-        <v>2779</v>
+        <v>2774</v>
       </c>
       <c r="C490" s="6" t="s">
-        <v>2779</v>
+        <v>2774</v>
       </c>
       <c r="D490" t="s">
-        <v>2780</v>
+        <v>2775</v>
       </c>
     </row>
     <row r="491" spans="1:4" hidden="1">
@@ -17234,13 +17282,13 @@
         <v>848</v>
       </c>
       <c r="B491" s="5" t="s">
-        <v>2781</v>
+        <v>2776</v>
       </c>
       <c r="C491" s="6" t="s">
-        <v>2781</v>
+        <v>2776</v>
       </c>
       <c r="D491" t="s">
-        <v>2782</v>
+        <v>2777</v>
       </c>
     </row>
     <row r="492" spans="1:4" hidden="1">
@@ -17248,13 +17296,13 @@
         <v>848</v>
       </c>
       <c r="B492" s="5" t="s">
-        <v>2784</v>
+        <v>2779</v>
       </c>
       <c r="C492" s="6" t="s">
-        <v>2784</v>
+        <v>2779</v>
       </c>
       <c r="D492" t="s">
-        <v>2783</v>
+        <v>2778</v>
       </c>
     </row>
     <row r="493" spans="1:4" hidden="1">
@@ -23664,13 +23712,13 @@
         <v>554</v>
       </c>
       <c r="B954" s="1" t="s">
-        <v>2822</v>
+        <v>2817</v>
       </c>
       <c r="C954" s="1" t="s">
-        <v>2822</v>
+        <v>2817</v>
       </c>
       <c r="D954" t="s">
-        <v>2823</v>
+        <v>2818</v>
       </c>
     </row>
     <row r="955" spans="1:4">
@@ -24059,7 +24107,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AB4C2C2-B1A2-4435-AA2E-590F77DA8D30}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:T110"/>
+  <dimension ref="A1:T112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.28515625" style="6" customWidth="1"/>
@@ -24133,7 +24181,7 @@
         <v>2563</v>
       </c>
       <c r="R1" s="39" t="s">
-        <v>2718</v>
+        <v>2716</v>
       </c>
       <c r="S1" s="39" t="s">
         <v>2450</v>
@@ -24290,13 +24338,13 @@
       </c>
       <c r="N5" s="29"/>
       <c r="O5" s="29" t="s">
-        <v>2795</v>
+        <v>2790</v>
       </c>
       <c r="P5" s="29" t="s">
-        <v>2726</v>
-      </c>
-      <c r="Q5" s="40" t="s">
-        <v>1891</v>
+        <v>2722</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>2835</v>
       </c>
       <c r="R5" s="40"/>
       <c r="S5" s="40"/>
@@ -24337,13 +24385,13 @@
       </c>
       <c r="N6" s="29"/>
       <c r="O6" s="29" t="s">
-        <v>2801</v>
+        <v>2796</v>
       </c>
       <c r="P6" s="29" t="s">
-        <v>2724</v>
-      </c>
-      <c r="Q6" s="40" t="s">
-        <v>1891</v>
+        <v>2720</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>2847</v>
       </c>
       <c r="R6" s="40"/>
       <c r="S6" s="40"/>
@@ -24384,13 +24432,13 @@
       </c>
       <c r="N7" s="29"/>
       <c r="O7" s="29" t="s">
-        <v>2793</v>
+        <v>2788</v>
       </c>
       <c r="P7" s="29" t="s">
-        <v>2729</v>
-      </c>
-      <c r="Q7" s="40" t="s">
-        <v>2689</v>
+        <v>2725</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>2845</v>
       </c>
       <c r="R7" s="40"/>
       <c r="S7" s="40"/>
@@ -24434,10 +24482,10 @@
         <v>2657</v>
       </c>
       <c r="P8" s="29" t="s">
-        <v>2736</v>
-      </c>
-      <c r="Q8" s="40" t="s">
-        <v>1891</v>
+        <v>2732</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>2839</v>
       </c>
       <c r="R8" s="40"/>
       <c r="S8" s="40"/>
@@ -24472,13 +24520,13 @@
       <c r="M9" s="29"/>
       <c r="N9" s="29"/>
       <c r="O9" s="29" t="s">
-        <v>2789</v>
+        <v>2784</v>
       </c>
       <c r="P9" s="29" t="s">
-        <v>2722</v>
-      </c>
-      <c r="Q9" s="40" t="s">
-        <v>1891</v>
+        <v>2718</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>2838</v>
       </c>
       <c r="R9" s="40"/>
       <c r="S9" s="40"/>
@@ -24522,10 +24570,10 @@
         <v>2643</v>
       </c>
       <c r="P10" s="29" t="s">
-        <v>2708</v>
+        <v>2706</v>
       </c>
       <c r="Q10" s="40" t="s">
-        <v>2690</v>
+        <v>2689</v>
       </c>
       <c r="R10" s="40"/>
       <c r="S10" s="40"/>
@@ -24562,13 +24610,13 @@
       <c r="M11" s="29"/>
       <c r="N11" s="29"/>
       <c r="O11" s="29" t="s">
-        <v>2810</v>
+        <v>2805</v>
       </c>
       <c r="P11" s="29" t="s">
-        <v>2728</v>
-      </c>
-      <c r="Q11" s="40" t="s">
-        <v>1891</v>
+        <v>2724</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>2843</v>
       </c>
       <c r="R11" s="40"/>
       <c r="S11" s="40"/>
@@ -24614,10 +24662,10 @@
         <v>2600</v>
       </c>
       <c r="P12" s="29" t="s">
-        <v>2709</v>
+        <v>2707</v>
       </c>
       <c r="Q12" s="40" t="s">
-        <v>2691</v>
+        <v>2690</v>
       </c>
       <c r="R12" s="40"/>
       <c r="S12" s="40"/>
@@ -24656,10 +24704,10 @@
       <c r="M13" s="29"/>
       <c r="N13" s="29"/>
       <c r="O13" s="29" t="s">
-        <v>2790</v>
+        <v>2785</v>
       </c>
       <c r="P13" s="29" t="s">
-        <v>2731</v>
+        <v>2727</v>
       </c>
       <c r="Q13" s="40" t="s">
         <v>1891</v>
@@ -24701,10 +24749,10 @@
       <c r="M14" s="29"/>
       <c r="N14" s="29"/>
       <c r="O14" s="29" t="s">
-        <v>2802</v>
+        <v>2797</v>
       </c>
       <c r="P14" s="29" t="s">
-        <v>2725</v>
+        <v>2721</v>
       </c>
       <c r="Q14" s="40" t="s">
         <v>1891</v>
@@ -24747,7 +24795,7 @@
         <v>2449</v>
       </c>
       <c r="Q15" s="41" t="s">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="R15" s="41"/>
       <c r="S15" s="41" t="s">
@@ -24826,7 +24874,7 @@
       <c r="N17" s="29"/>
       <c r="O17" s="29"/>
       <c r="P17" s="29" t="s">
-        <v>2710</v>
+        <v>2708</v>
       </c>
       <c r="Q17" s="40" t="s">
         <v>1891</v>
@@ -24912,10 +24960,10 @@
       <c r="N19" s="29"/>
       <c r="O19" s="29"/>
       <c r="P19" s="29" t="s">
-        <v>2711</v>
+        <v>2709</v>
       </c>
       <c r="Q19" s="40" t="s">
-        <v>2693</v>
+        <v>2692</v>
       </c>
       <c r="R19" s="40"/>
       <c r="S19" s="40"/>
@@ -24952,15 +25000,17 @@
       <c r="M20" s="29"/>
       <c r="N20" s="29"/>
       <c r="O20" s="29" t="s">
-        <v>2792</v>
+        <v>2787</v>
       </c>
       <c r="P20" s="29" t="s">
         <v>2469</v>
       </c>
       <c r="Q20" s="40" t="s">
-        <v>2750</v>
-      </c>
-      <c r="R20" s="40"/>
+        <v>2746</v>
+      </c>
+      <c r="R20" t="s">
+        <v>2846</v>
+      </c>
       <c r="S20" s="40"/>
       <c r="T20" s="33" t="str">
         <f t="shared" si="0"/>
@@ -24999,13 +25049,13 @@
         <v>2468</v>
       </c>
       <c r="Q21" s="40" t="s">
-        <v>2694</v>
-      </c>
-      <c r="R21" s="40" t="s">
-        <v>2720</v>
+        <v>2693</v>
+      </c>
+      <c r="R21" t="s">
+        <v>2844</v>
       </c>
       <c r="S21" s="40" t="s">
-        <v>2813</v>
+        <v>2808</v>
       </c>
       <c r="T21" s="33" t="str">
         <f t="shared" si="0"/>
@@ -25045,7 +25095,7 @@
       </c>
       <c r="O22" s="29"/>
       <c r="P22" s="29" t="s">
-        <v>2747</v>
+        <v>2743</v>
       </c>
       <c r="Q22" s="40" t="s">
         <v>1891</v>
@@ -25111,7 +25161,7 @@
       </c>
       <c r="P24" s="29"/>
       <c r="Q24" s="40" t="s">
-        <v>2717</v>
+        <v>2715</v>
       </c>
       <c r="R24" s="40"/>
       <c r="S24" s="40"/>
@@ -25146,10 +25196,10 @@
       <c r="M25" s="29"/>
       <c r="N25" s="29"/>
       <c r="O25" s="29" t="s">
-        <v>2807</v>
+        <v>2802</v>
       </c>
       <c r="P25" s="29" t="s">
-        <v>2723</v>
+        <v>2719</v>
       </c>
       <c r="Q25" s="40" t="s">
         <v>1891</v>
@@ -25325,7 +25375,7 @@
       <c r="E30" s="58"/>
       <c r="F30" s="45"/>
       <c r="G30" s="75" t="s">
-        <v>2788</v>
+        <v>2783</v>
       </c>
       <c r="H30" s="45"/>
       <c r="I30" s="45"/>
@@ -25342,10 +25392,10 @@
         <v>2599</v>
       </c>
       <c r="P30" s="29" t="s">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="Q30" s="40" t="s">
-        <v>2695</v>
+        <v>2694</v>
       </c>
       <c r="R30" s="40"/>
       <c r="S30" s="40"/>
@@ -25381,12 +25431,14 @@
       <c r="N31" s="29"/>
       <c r="O31" s="29"/>
       <c r="P31" s="29" t="s">
-        <v>2721</v>
+        <v>2717</v>
       </c>
       <c r="Q31" s="40" t="s">
-        <v>2791</v>
-      </c>
-      <c r="R31" s="40"/>
+        <v>2786</v>
+      </c>
+      <c r="R31" t="s">
+        <v>2841</v>
+      </c>
       <c r="S31" s="40"/>
       <c r="T31" s="33" t="str">
         <f t="shared" si="1"/>
@@ -25425,7 +25477,7 @@
       <c r="O32" s="29"/>
       <c r="P32" s="29"/>
       <c r="Q32" s="40" t="s">
-        <v>2696</v>
+        <v>2695</v>
       </c>
       <c r="R32" s="40"/>
       <c r="S32" s="40"/>
@@ -25460,10 +25512,10 @@
       <c r="M33" s="29"/>
       <c r="N33" s="29"/>
       <c r="O33" s="29" t="s">
-        <v>2797</v>
+        <v>2792</v>
       </c>
       <c r="P33" s="29" t="s">
-        <v>2743</v>
+        <v>2739</v>
       </c>
       <c r="Q33" s="40" t="s">
         <v>1891</v>
@@ -25623,10 +25675,10 @@
       <c r="N37" s="29"/>
       <c r="O37" s="29"/>
       <c r="P37" s="29" t="s">
-        <v>2713</v>
+        <v>2711</v>
       </c>
       <c r="Q37" s="40" t="s">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="R37" s="40"/>
       <c r="S37" s="40"/>
@@ -25666,10 +25718,10 @@
       <c r="N38" s="29"/>
       <c r="O38" s="29"/>
       <c r="P38" s="29" t="s">
-        <v>2714</v>
+        <v>2712</v>
       </c>
       <c r="Q38" s="40" t="s">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="R38" s="40"/>
       <c r="S38" s="40"/>
@@ -25710,10 +25762,10 @@
         <v>8936156732859</v>
       </c>
       <c r="O39" s="29" t="s">
-        <v>2796</v>
+        <v>2791</v>
       </c>
       <c r="P39" s="29" t="s">
-        <v>2741</v>
+        <v>2737</v>
       </c>
       <c r="Q39" s="40" t="s">
         <v>2687</v>
@@ -25780,7 +25832,7 @@
       <c r="N41" s="29"/>
       <c r="O41" s="29"/>
       <c r="P41" s="29" t="s">
-        <v>2742</v>
+        <v>2738</v>
       </c>
       <c r="Q41" s="40" t="s">
         <v>1891</v>
@@ -25825,13 +25877,13 @@
         <v>2641</v>
       </c>
       <c r="P42" s="29" t="s">
-        <v>2806</v>
-      </c>
-      <c r="Q42" s="40" t="s">
-        <v>2699</v>
+        <v>2801</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>2848</v>
       </c>
       <c r="R42" s="40" t="s">
-        <v>2814</v>
+        <v>2809</v>
       </c>
       <c r="S42" s="40"/>
       <c r="T42" s="33" t="str">
@@ -25914,7 +25966,7 @@
         <v>2499</v>
       </c>
       <c r="Q44" s="40" t="s">
-        <v>2749</v>
+        <v>2745</v>
       </c>
       <c r="R44" s="40"/>
       <c r="S44" s="40"/>
@@ -25988,13 +26040,13 @@
       <c r="M46" s="29"/>
       <c r="N46" s="29"/>
       <c r="O46" s="29" t="s">
-        <v>2799</v>
+        <v>2794</v>
       </c>
       <c r="P46" s="29" t="s">
-        <v>2715</v>
+        <v>2713</v>
       </c>
       <c r="Q46" s="40" t="s">
-        <v>2700</v>
+        <v>2698</v>
       </c>
       <c r="R46" s="40"/>
       <c r="S46" s="40"/>
@@ -26032,10 +26084,10 @@
         <v>2640</v>
       </c>
       <c r="P47" s="29" t="s">
-        <v>2737</v>
-      </c>
-      <c r="Q47" s="40" t="s">
-        <v>1891</v>
+        <v>2733</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>2837</v>
       </c>
       <c r="R47" s="40"/>
       <c r="S47" s="40"/>
@@ -26077,13 +26129,13 @@
         <v>2633</v>
       </c>
       <c r="P48" s="29" t="s">
-        <v>2805</v>
+        <v>2800</v>
       </c>
       <c r="Q48" s="29" t="s">
-        <v>2701</v>
-      </c>
-      <c r="R48" s="29" t="s">
-        <v>2719</v>
+        <v>2699</v>
+      </c>
+      <c r="R48" t="s">
+        <v>2840</v>
       </c>
       <c r="S48" s="43" t="s">
         <v>2451</v>
@@ -26191,12 +26243,14 @@
         <v>2658</v>
       </c>
       <c r="P51" s="67" t="s">
-        <v>2727</v>
+        <v>2723</v>
       </c>
       <c r="Q51" s="41" t="s">
-        <v>2702</v>
-      </c>
-      <c r="R51" s="41"/>
+        <v>2700</v>
+      </c>
+      <c r="R51" t="s">
+        <v>2834</v>
+      </c>
     </row>
     <row r="52" spans="1:20">
       <c r="A52" s="6" t="s">
@@ -26264,13 +26318,13 @@
       <c r="H54" s="47"/>
       <c r="I54" s="47"/>
       <c r="O54" s="30" t="s">
-        <v>2798</v>
+        <v>2793</v>
       </c>
       <c r="P54" s="67" t="s">
         <v>2437</v>
       </c>
       <c r="Q54" s="41" t="s">
-        <v>2703</v>
+        <v>2701</v>
       </c>
       <c r="R54" s="41"/>
     </row>
@@ -26459,10 +26513,10 @@
       <c r="E62" s="60"/>
       <c r="G62" s="46"/>
       <c r="O62" s="30" t="s">
-        <v>2794</v>
+        <v>2789</v>
       </c>
       <c r="P62" s="67" t="s">
-        <v>2735</v>
+        <v>2731</v>
       </c>
       <c r="Q62" s="41" t="s">
         <v>1891</v>
@@ -26485,13 +26539,13 @@
       <c r="E63" s="60"/>
       <c r="G63" s="46"/>
       <c r="O63" s="30" t="s">
-        <v>2804</v>
+        <v>2799</v>
       </c>
       <c r="P63" s="67" t="s">
         <v>2445</v>
       </c>
       <c r="Q63" s="41" t="s">
-        <v>2704</v>
+        <v>2702</v>
       </c>
       <c r="R63" s="41"/>
       <c r="S63" s="41" t="s">
@@ -26515,10 +26569,10 @@
       <c r="G64" s="46"/>
       <c r="O64" s="30"/>
       <c r="P64" s="67" t="s">
-        <v>2716</v>
+        <v>2714</v>
       </c>
       <c r="Q64" s="41" t="s">
-        <v>2705</v>
+        <v>2703</v>
       </c>
       <c r="R64" s="41"/>
       <c r="S64" s="41" t="s">
@@ -26541,10 +26595,10 @@
       <c r="E65" s="60"/>
       <c r="G65" s="46"/>
       <c r="O65" s="30" t="s">
-        <v>2800</v>
+        <v>2795</v>
       </c>
       <c r="P65" s="67" t="s">
-        <v>2734</v>
+        <v>2730</v>
       </c>
       <c r="Q65" s="41" t="s">
         <v>1891</v>
@@ -26567,10 +26621,10 @@
       <c r="E66" s="60"/>
       <c r="G66" s="46"/>
       <c r="O66" s="30" t="s">
-        <v>2803</v>
+        <v>2798</v>
       </c>
       <c r="P66" s="67" t="s">
-        <v>2744</v>
+        <v>2740</v>
       </c>
       <c r="Q66" s="41" t="s">
         <v>1891</v>
@@ -26594,7 +26648,7 @@
       <c r="G67" s="46"/>
       <c r="O67" s="30"/>
       <c r="P67" s="67" t="s">
-        <v>2739</v>
+        <v>2735</v>
       </c>
       <c r="Q67" s="41" t="s">
         <v>1891</v>
@@ -26618,10 +26672,10 @@
       <c r="G68" s="46"/>
       <c r="O68" s="30"/>
       <c r="P68" s="67" t="s">
-        <v>2738</v>
-      </c>
-      <c r="Q68" s="41" t="s">
-        <v>1891</v>
+        <v>2734</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>2842</v>
       </c>
       <c r="R68" s="41"/>
     </row>
@@ -26666,10 +26720,10 @@
         <v>2630</v>
       </c>
       <c r="P70" s="67" t="s">
-        <v>2740</v>
+        <v>2736</v>
       </c>
       <c r="Q70" s="67" t="s">
-        <v>2812</v>
+        <v>2807</v>
       </c>
       <c r="R70" s="41"/>
     </row>
@@ -26690,7 +26744,7 @@
       <c r="G71" s="46"/>
       <c r="O71" s="30"/>
       <c r="P71" s="67" t="s">
-        <v>2754</v>
+        <v>2749</v>
       </c>
       <c r="Q71" s="41" t="s">
         <v>1891</v>
@@ -26714,7 +26768,7 @@
       <c r="G72" s="46"/>
       <c r="O72" s="30"/>
       <c r="P72" s="67" t="s">
-        <v>2748</v>
+        <v>2744</v>
       </c>
       <c r="Q72" s="41"/>
       <c r="R72" s="41"/>
@@ -26744,7 +26798,7 @@
       <c r="N73" s="37"/>
       <c r="O73" s="37"/>
       <c r="P73" s="68" t="s">
-        <v>2730</v>
+        <v>2726</v>
       </c>
       <c r="Q73" s="42" t="s">
         <v>1891</v>
@@ -26778,7 +26832,7 @@
       <c r="N74" s="37"/>
       <c r="O74" s="37"/>
       <c r="P74" s="74" t="s">
-        <v>2732</v>
+        <v>2728</v>
       </c>
       <c r="Q74" s="42" t="s">
         <v>1891</v>
@@ -26861,9 +26915,11 @@
         <v>3201891</v>
       </c>
       <c r="O76" s="37"/>
-      <c r="P76" s="68"/>
+      <c r="P76" t="s">
+        <v>2836</v>
+      </c>
       <c r="Q76" s="42" t="s">
-        <v>2706</v>
+        <v>2704</v>
       </c>
       <c r="R76" s="42"/>
       <c r="S76" s="42"/>
@@ -27105,12 +27161,14 @@
       <c r="G84" s="46"/>
       <c r="O84" s="30"/>
       <c r="P84" s="67" t="s">
-        <v>2808</v>
+        <v>2803</v>
       </c>
       <c r="Q84" s="41" t="s">
-        <v>2707</v>
-      </c>
-      <c r="R84" s="41"/>
+        <v>2705</v>
+      </c>
+      <c r="R84" t="s">
+        <v>2849</v>
+      </c>
     </row>
     <row r="85" spans="1:20">
       <c r="A85" s="12" t="s">
@@ -27242,7 +27300,9 @@
       <c r="G89" s="48"/>
       <c r="H89" s="48"/>
       <c r="I89" s="48"/>
-      <c r="J89" s="12"/>
+      <c r="J89" s="12">
+        <v>3622987</v>
+      </c>
       <c r="K89" s="37">
         <v>8936156732767</v>
       </c>
@@ -27500,10 +27560,10 @@
     </row>
     <row r="99" spans="1:20">
       <c r="A99" s="6" t="s">
-        <v>2745</v>
+        <v>2741</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>2746</v>
+        <v>2742</v>
       </c>
       <c r="C99" s="46"/>
       <c r="D99" s="70"/>
@@ -27516,15 +27576,22 @@
     </row>
     <row r="100" spans="1:20">
       <c r="A100" t="s">
-        <v>2752</v>
+        <v>2748</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>2753</v>
-      </c>
-      <c r="C100" s="46"/>
-      <c r="D100" s="70"/>
+        <v>2850</v>
+      </c>
+      <c r="C100" s="46">
+        <v>0.31</v>
+      </c>
+      <c r="D100" s="70">
+        <v>36</v>
+      </c>
       <c r="E100" s="46"/>
       <c r="G100" s="46"/>
+      <c r="J100" s="6">
+        <v>3622988</v>
+      </c>
       <c r="O100" s="30"/>
       <c r="P100" s="67"/>
       <c r="Q100" s="41"/>
@@ -27532,10 +27599,10 @@
     </row>
     <row r="101" spans="1:20">
       <c r="A101" s="6" t="s">
-        <v>2759</v>
+        <v>2754</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>2758</v>
+        <v>2753</v>
       </c>
       <c r="C101" s="46"/>
       <c r="D101" s="70"/>
@@ -27548,10 +27615,10 @@
     </row>
     <row r="102" spans="1:20">
       <c r="A102" s="6" t="s">
-        <v>2760</v>
+        <v>2755</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>2761</v>
+        <v>2756</v>
       </c>
       <c r="C102" s="46">
         <v>10</v>
@@ -27566,10 +27633,10 @@
     </row>
     <row r="103" spans="1:20">
       <c r="A103" s="10" t="s">
-        <v>2762</v>
+        <v>2757</v>
       </c>
       <c r="B103" s="10" t="s">
-        <v>2763</v>
+        <v>2758</v>
       </c>
       <c r="C103" s="46">
         <v>10</v>
@@ -27587,10 +27654,10 @@
     </row>
     <row r="104" spans="1:20">
       <c r="A104" s="10" t="s">
-        <v>2764</v>
+        <v>2759</v>
       </c>
       <c r="B104" s="10" t="s">
-        <v>2765</v>
+        <v>2760</v>
       </c>
       <c r="C104" s="46">
         <v>10</v>
@@ -27608,10 +27675,10 @@
     </row>
     <row r="105" spans="1:20">
       <c r="A105" s="10" t="s">
-        <v>2766</v>
+        <v>2761</v>
       </c>
       <c r="B105" s="10" t="s">
-        <v>2767</v>
+        <v>2762</v>
       </c>
       <c r="C105" s="46">
         <v>10</v>
@@ -27629,10 +27696,10 @@
     </row>
     <row r="106" spans="1:20">
       <c r="A106" s="10" t="s">
-        <v>2768</v>
+        <v>2763</v>
       </c>
       <c r="B106" s="10" t="s">
-        <v>2769</v>
+        <v>2764</v>
       </c>
       <c r="C106" s="46">
         <v>10</v>
@@ -27650,10 +27717,10 @@
     </row>
     <row r="107" spans="1:20">
       <c r="A107" s="10" t="s">
-        <v>2770</v>
+        <v>2765</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>2771</v>
+        <v>2766</v>
       </c>
       <c r="C107" s="46">
         <v>10</v>
@@ -27671,10 +27738,10 @@
     </row>
     <row r="108" spans="1:20">
       <c r="A108" s="10" t="s">
-        <v>2772</v>
+        <v>2767</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>2773</v>
+        <v>2768</v>
       </c>
       <c r="C108" s="46">
         <v>10</v>
@@ -27692,18 +27759,34 @@
     </row>
     <row r="109" spans="1:20">
       <c r="A109" s="6" t="s">
-        <v>2817</v>
+        <v>2812</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>2818</v>
+        <v>2813</v>
       </c>
     </row>
     <row r="110" spans="1:20">
       <c r="A110" s="6" t="s">
-        <v>2824</v>
+        <v>2819</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>2825</v>
+        <v>2820</v>
+      </c>
+    </row>
+    <row r="111" spans="1:20">
+      <c r="A111" t="s">
+        <v>2830</v>
+      </c>
+      <c r="B111" s="6" t="s">
+        <v>2831</v>
+      </c>
+    </row>
+    <row r="112" spans="1:20">
+      <c r="A112" t="s">
+        <v>2832</v>
+      </c>
+      <c r="B112" s="6" t="s">
+        <v>2833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>